<commit_message>
rating appearance for range field
</commit_message>
<xml_diff>
--- a/formats/testdata/noformulas.xlsx
+++ b/formats/testdata/noformulas.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="77">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t xml:space="preserve">start=3 end=30 step=6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rating</t>
   </si>
   <si>
     <t xml:space="preserve">text</t>
@@ -460,159 +463,162 @@
       <c r="I7" s="0" t="s">
         <v>24</v>
       </c>
+      <c r="J7" s="0" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>18</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="J18" s="0" t="s">
         <v>47</v>
-      </c>
-      <c r="J18" s="0" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -620,10 +626,10 @@
         <v>13</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>18</v>
@@ -631,32 +637,32 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -684,7 +690,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>1</v>
@@ -695,35 +701,35 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -747,26 +753,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>